<commit_message>
update import & export file
</commit_message>
<xml_diff>
--- a/backend/InternLink/InternLink.API/Templates/InternshipExportTemplate.xlsx
+++ b/backend/InternLink/InternLink.API/Templates/InternshipExportTemplate.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Downloads\internlink\frontend\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Downloads\internlink\backend\InternLink\InternLink.API\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15C498C5-4A23-4498-9CE3-0C0DD5669405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40246DB6-113B-46F6-9C0E-652E9D0F9F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DANH SÁCH (2)" sheetId="4" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="178">
   <si>
     <t>STT</t>
   </si>
@@ -575,13 +575,16 @@
   </si>
   <si>
     <t>kết quả</t>
+  </si>
+  <si>
+    <t>DANH SÁCH SINH VIÊN THỰC TẬP TẠI DOANH NGHIỆP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="26">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -691,13 +694,6 @@
       <family val="1"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -712,12 +708,6 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="13"/>
-      <color rgb="FF0070C0"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -748,6 +738,48 @@
     <font>
       <sz val="11"/>
       <name val="VNI-Times"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="163"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="163"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF0070C0"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="163"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF081B3A"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="163"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="163"/>
+      <scheme val="major"/>
     </font>
   </fonts>
   <fills count="7">
@@ -865,12 +897,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -959,53 +991,35 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1017,31 +1031,76 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1336,35 +1395,35 @@
     <col min="8" max="8" width="18.69921875" style="16" customWidth="1"/>
     <col min="9" max="12" width="16.3984375" customWidth="1"/>
     <col min="13" max="13" width="10.09765625" customWidth="1"/>
-    <col min="14" max="14" width="8.69921875" style="45" customWidth="1"/>
-    <col min="15" max="20" width="8.69921875" style="46" customWidth="1"/>
-    <col min="21" max="21" width="25.09765625" style="43" customWidth="1"/>
+    <col min="14" max="14" width="8.69921875" style="39" customWidth="1"/>
+    <col min="15" max="20" width="8.69921875" style="40" customWidth="1"/>
+    <col min="21" max="21" width="25.09765625" style="37" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" s="3" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
-      <c r="P1" s="56"/>
-      <c r="Q1" s="56"/>
-      <c r="R1" s="56"/>
-      <c r="S1" s="56"/>
-      <c r="T1" s="56"/>
-      <c r="U1" s="56"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
+      <c r="M1" s="50"/>
+      <c r="N1" s="50"/>
+      <c r="O1" s="50"/>
+      <c r="P1" s="50"/>
+      <c r="Q1" s="50"/>
+      <c r="R1" s="50"/>
+      <c r="S1" s="50"/>
+      <c r="T1" s="50"/>
+      <c r="U1" s="50"/>
     </row>
     <row r="2" spans="1:21" ht="35.85" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -1379,7 +1438,7 @@
       <c r="D2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="33" t="s">
+      <c r="E2" s="31" t="s">
         <v>3</v>
       </c>
       <c r="F2" s="29" t="s">
@@ -1394,16 +1453,16 @@
       <c r="I2" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="J2" s="47" t="s">
+      <c r="J2" s="41" t="s">
         <v>154</v>
       </c>
-      <c r="K2" s="47" t="s">
+      <c r="K2" s="41" t="s">
         <v>156</v>
       </c>
-      <c r="L2" s="49" t="s">
+      <c r="L2" s="43" t="s">
         <v>157</v>
       </c>
-      <c r="M2" s="33" t="s">
+      <c r="M2" s="31" t="s">
         <v>34</v>
       </c>
       <c r="N2" s="29" t="s">
@@ -1441,12 +1500,12 @@
       <c r="G3" s="4"/>
       <c r="H3" s="10"/>
       <c r="I3" s="4"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="48">
+      <c r="J3" s="42"/>
+      <c r="K3" s="42">
         <f>I3*0.4+J3*0.6</f>
         <v>0</v>
       </c>
-      <c r="L3" s="48" t="str">
+      <c r="L3" s="42" t="str">
         <f t="shared" ref="L3:L34" si="0">VLOOKUP(K3,$I$64:$L$71,4,1)</f>
         <v>không thực tập</v>
       </c>
@@ -1473,12 +1532,12 @@
       <c r="G4" s="4"/>
       <c r="H4" s="10"/>
       <c r="I4" s="4"/>
-      <c r="J4" s="48"/>
-      <c r="K4" s="48">
+      <c r="J4" s="42"/>
+      <c r="K4" s="42">
         <f>I4*0.4+J4*0.6</f>
         <v>0</v>
       </c>
-      <c r="L4" s="48" t="str">
+      <c r="L4" s="42" t="str">
         <f>VLOOKUP(K4,$I$64:$L$71,4,1)</f>
         <v>không thực tập</v>
       </c>
@@ -1505,12 +1564,12 @@
       <c r="G5" s="4"/>
       <c r="H5" s="10"/>
       <c r="I5" s="4"/>
-      <c r="J5" s="48"/>
-      <c r="K5" s="48">
-        <f t="shared" ref="K4:K52" si="2">I5*0.4+J5*0.6</f>
-        <v>0</v>
-      </c>
-      <c r="L5" s="48" t="str">
+      <c r="J5" s="42"/>
+      <c r="K5" s="42">
+        <f t="shared" ref="K5:K52" si="2">I5*0.4+J5*0.6</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -1537,12 +1596,12 @@
       <c r="G6" s="4"/>
       <c r="H6" s="10"/>
       <c r="I6" s="4"/>
-      <c r="J6" s="48"/>
-      <c r="K6" s="48">
+      <c r="J6" s="42"/>
+      <c r="K6" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L6" s="48" t="str">
+      <c r="L6" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -1569,12 +1628,12 @@
       <c r="G7" s="4"/>
       <c r="H7" s="10"/>
       <c r="I7" s="4"/>
-      <c r="J7" s="48"/>
-      <c r="K7" s="48">
+      <c r="J7" s="42"/>
+      <c r="K7" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L7" s="48" t="str">
+      <c r="L7" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -1601,12 +1660,12 @@
       <c r="G8" s="4"/>
       <c r="H8" s="14"/>
       <c r="I8" s="4"/>
-      <c r="J8" s="48"/>
-      <c r="K8" s="48">
+      <c r="J8" s="42"/>
+      <c r="K8" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L8" s="48" t="str">
+      <c r="L8" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -1633,12 +1692,12 @@
       <c r="G9" s="4"/>
       <c r="H9" s="10"/>
       <c r="I9" s="4"/>
-      <c r="J9" s="48"/>
-      <c r="K9" s="48">
+      <c r="J9" s="42"/>
+      <c r="K9" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L9" s="48" t="str">
+      <c r="L9" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -1665,12 +1724,12 @@
       <c r="G10" s="4"/>
       <c r="H10" s="10"/>
       <c r="I10" s="4"/>
-      <c r="J10" s="48"/>
-      <c r="K10" s="48">
+      <c r="J10" s="42"/>
+      <c r="K10" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L10" s="48" t="str">
+      <c r="L10" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -1697,12 +1756,12 @@
       <c r="G11" s="4"/>
       <c r="H11" s="10"/>
       <c r="I11" s="4"/>
-      <c r="J11" s="48"/>
-      <c r="K11" s="48">
+      <c r="J11" s="42"/>
+      <c r="K11" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L11" s="48" t="str">
+      <c r="L11" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -1729,12 +1788,12 @@
       <c r="G12" s="4"/>
       <c r="H12" s="10"/>
       <c r="I12" s="4"/>
-      <c r="J12" s="48"/>
-      <c r="K12" s="48">
+      <c r="J12" s="42"/>
+      <c r="K12" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L12" s="48" t="str">
+      <c r="L12" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -1761,12 +1820,12 @@
       <c r="G13" s="4"/>
       <c r="H13" s="10"/>
       <c r="I13" s="4"/>
-      <c r="J13" s="48"/>
-      <c r="K13" s="48">
+      <c r="J13" s="42"/>
+      <c r="K13" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L13" s="48" t="str">
+      <c r="L13" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -1793,12 +1852,12 @@
       <c r="G14" s="4"/>
       <c r="H14" s="10"/>
       <c r="I14" s="4"/>
-      <c r="J14" s="48"/>
-      <c r="K14" s="48">
+      <c r="J14" s="42"/>
+      <c r="K14" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L14" s="48" t="str">
+      <c r="L14" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -1825,12 +1884,12 @@
       <c r="G15" s="4"/>
       <c r="H15" s="10"/>
       <c r="I15" s="4"/>
-      <c r="J15" s="48"/>
-      <c r="K15" s="48">
+      <c r="J15" s="42"/>
+      <c r="K15" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L15" s="48" t="str">
+      <c r="L15" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -1857,12 +1916,12 @@
       <c r="G16" s="4"/>
       <c r="H16" s="10"/>
       <c r="I16" s="4"/>
-      <c r="J16" s="48"/>
-      <c r="K16" s="48">
+      <c r="J16" s="42"/>
+      <c r="K16" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L16" s="48" t="str">
+      <c r="L16" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -1889,12 +1948,12 @@
       <c r="G17" s="4"/>
       <c r="H17" s="10"/>
       <c r="I17" s="4"/>
-      <c r="J17" s="48"/>
-      <c r="K17" s="48">
+      <c r="J17" s="42"/>
+      <c r="K17" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L17" s="48" t="str">
+      <c r="L17" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -1921,12 +1980,12 @@
       <c r="G18" s="4"/>
       <c r="H18" s="10"/>
       <c r="I18" s="4"/>
-      <c r="J18" s="48"/>
-      <c r="K18" s="48">
+      <c r="J18" s="42"/>
+      <c r="K18" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L18" s="48" t="str">
+      <c r="L18" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -1948,17 +2007,17 @@
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
-      <c r="E19" s="32"/>
+      <c r="E19" s="30"/>
       <c r="F19" s="13"/>
       <c r="G19" s="4"/>
       <c r="H19" s="10"/>
       <c r="I19" s="4"/>
-      <c r="J19" s="48"/>
-      <c r="K19" s="48">
+      <c r="J19" s="42"/>
+      <c r="K19" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L19" s="48" t="str">
+      <c r="L19" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -1985,12 +2044,12 @@
       <c r="G20" s="4"/>
       <c r="H20" s="10"/>
       <c r="I20" s="4"/>
-      <c r="J20" s="48"/>
-      <c r="K20" s="48">
+      <c r="J20" s="42"/>
+      <c r="K20" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L20" s="48" t="str">
+      <c r="L20" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -2017,12 +2076,12 @@
       <c r="G21" s="4"/>
       <c r="H21" s="10"/>
       <c r="I21" s="4"/>
-      <c r="J21" s="48"/>
-      <c r="K21" s="48">
+      <c r="J21" s="42"/>
+      <c r="K21" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L21" s="48" t="str">
+      <c r="L21" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -2044,17 +2103,17 @@
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
-      <c r="E22" s="34"/>
+      <c r="E22" s="32"/>
       <c r="F22" s="13"/>
       <c r="G22" s="4"/>
       <c r="H22" s="10"/>
       <c r="I22" s="4"/>
-      <c r="J22" s="48"/>
-      <c r="K22" s="48">
+      <c r="J22" s="42"/>
+      <c r="K22" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L22" s="48" t="str">
+      <c r="L22" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -2081,12 +2140,12 @@
       <c r="G23" s="4"/>
       <c r="H23" s="10"/>
       <c r="I23" s="4"/>
-      <c r="J23" s="48"/>
-      <c r="K23" s="48">
+      <c r="J23" s="42"/>
+      <c r="K23" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L23" s="48" t="str">
+      <c r="L23" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -2108,17 +2167,17 @@
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
-      <c r="E24" s="32"/>
+      <c r="E24" s="30"/>
       <c r="F24" s="13"/>
       <c r="G24" s="4"/>
       <c r="H24" s="10"/>
       <c r="I24" s="4"/>
-      <c r="J24" s="48"/>
-      <c r="K24" s="48">
+      <c r="J24" s="42"/>
+      <c r="K24" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L24" s="48" t="str">
+      <c r="L24" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -2145,12 +2204,12 @@
       <c r="G25" s="4"/>
       <c r="H25" s="10"/>
       <c r="I25" s="4"/>
-      <c r="J25" s="48"/>
-      <c r="K25" s="48">
+      <c r="J25" s="42"/>
+      <c r="K25" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L25" s="48" t="str">
+      <c r="L25" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -2177,12 +2236,12 @@
       <c r="G26" s="4"/>
       <c r="H26" s="10"/>
       <c r="I26" s="4"/>
-      <c r="J26" s="48"/>
-      <c r="K26" s="48">
+      <c r="J26" s="42"/>
+      <c r="K26" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L26" s="48" t="str">
+      <c r="L26" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -2209,12 +2268,12 @@
       <c r="G27" s="4"/>
       <c r="H27" s="10"/>
       <c r="I27" s="4"/>
-      <c r="J27" s="48"/>
-      <c r="K27" s="48">
+      <c r="J27" s="42"/>
+      <c r="K27" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L27" s="48" t="str">
+      <c r="L27" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -2241,12 +2300,12 @@
       <c r="G28" s="4"/>
       <c r="H28" s="10"/>
       <c r="I28" s="4"/>
-      <c r="J28" s="48"/>
-      <c r="K28" s="48">
+      <c r="J28" s="42"/>
+      <c r="K28" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L28" s="48" t="str">
+      <c r="L28" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -2273,12 +2332,12 @@
       <c r="G29" s="4"/>
       <c r="H29" s="10"/>
       <c r="I29" s="4"/>
-      <c r="J29" s="48"/>
-      <c r="K29" s="48">
+      <c r="J29" s="42"/>
+      <c r="K29" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L29" s="48" t="str">
+      <c r="L29" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -2305,12 +2364,12 @@
       <c r="G30" s="4"/>
       <c r="H30" s="10"/>
       <c r="I30" s="4"/>
-      <c r="J30" s="48"/>
-      <c r="K30" s="48">
+      <c r="J30" s="42"/>
+      <c r="K30" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L30" s="48" t="str">
+      <c r="L30" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -2337,12 +2396,12 @@
       <c r="G31" s="4"/>
       <c r="H31" s="10"/>
       <c r="I31" s="4"/>
-      <c r="J31" s="48"/>
-      <c r="K31" s="48">
+      <c r="J31" s="42"/>
+      <c r="K31" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L31" s="48" t="str">
+      <c r="L31" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -2369,12 +2428,12 @@
       <c r="G32" s="4"/>
       <c r="H32" s="10"/>
       <c r="I32" s="4"/>
-      <c r="J32" s="48"/>
-      <c r="K32" s="48">
+      <c r="J32" s="42"/>
+      <c r="K32" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L32" s="48" t="str">
+      <c r="L32" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -2401,12 +2460,12 @@
       <c r="G33" s="4"/>
       <c r="H33" s="10"/>
       <c r="I33" s="4"/>
-      <c r="J33" s="48"/>
-      <c r="K33" s="48">
+      <c r="J33" s="42"/>
+      <c r="K33" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L33" s="48" t="str">
+      <c r="L33" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -2433,12 +2492,12 @@
       <c r="G34" s="25"/>
       <c r="H34" s="15"/>
       <c r="I34" s="4"/>
-      <c r="J34" s="48"/>
-      <c r="K34" s="48">
+      <c r="J34" s="42"/>
+      <c r="K34" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L34" s="48" t="str">
+      <c r="L34" s="42" t="str">
         <f t="shared" si="0"/>
         <v>không thực tập</v>
       </c>
@@ -2465,12 +2524,12 @@
       <c r="G35" s="4"/>
       <c r="H35" s="10"/>
       <c r="I35" s="4"/>
-      <c r="J35" s="48"/>
-      <c r="K35" s="48">
+      <c r="J35" s="42"/>
+      <c r="K35" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L35" s="48" t="str">
+      <c r="L35" s="42" t="str">
         <f t="shared" ref="L35:L52" si="3">VLOOKUP(K35,$I$64:$L$71,4,1)</f>
         <v>không thực tập</v>
       </c>
@@ -2497,16 +2556,16 @@
       <c r="G36" s="26"/>
       <c r="H36" s="14"/>
       <c r="I36" s="4"/>
-      <c r="J36" s="48"/>
-      <c r="K36" s="48">
+      <c r="J36" s="42"/>
+      <c r="K36" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L36" s="48" t="str">
+      <c r="L36" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
-      <c r="M36" s="44"/>
+      <c r="M36" s="38"/>
       <c r="N36" s="7"/>
       <c r="O36" s="7"/>
       <c r="P36" s="7"/>
@@ -2529,16 +2588,16 @@
       <c r="G37" s="26"/>
       <c r="H37" s="10"/>
       <c r="I37" s="4"/>
-      <c r="J37" s="48"/>
-      <c r="K37" s="48">
+      <c r="J37" s="42"/>
+      <c r="K37" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L37" s="48" t="str">
+      <c r="L37" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
-      <c r="M37" s="44"/>
+      <c r="M37" s="38"/>
       <c r="N37" s="7"/>
       <c r="O37" s="7"/>
       <c r="P37" s="7"/>
@@ -2561,12 +2620,12 @@
       <c r="G38" s="4"/>
       <c r="H38" s="10"/>
       <c r="I38" s="4"/>
-      <c r="J38" s="48"/>
-      <c r="K38" s="48">
+      <c r="J38" s="42"/>
+      <c r="K38" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L38" s="48" t="str">
+      <c r="L38" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
@@ -2593,12 +2652,12 @@
       <c r="G39" s="4"/>
       <c r="H39" s="10"/>
       <c r="I39" s="4"/>
-      <c r="J39" s="48"/>
-      <c r="K39" s="48">
+      <c r="J39" s="42"/>
+      <c r="K39" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L39" s="48" t="str">
+      <c r="L39" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
@@ -2625,12 +2684,12 @@
       <c r="G40" s="4"/>
       <c r="H40" s="10"/>
       <c r="I40" s="4"/>
-      <c r="J40" s="48"/>
-      <c r="K40" s="48">
+      <c r="J40" s="42"/>
+      <c r="K40" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L40" s="48" t="str">
+      <c r="L40" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
@@ -2657,12 +2716,12 @@
       <c r="G41" s="4"/>
       <c r="H41" s="10"/>
       <c r="I41" s="4"/>
-      <c r="J41" s="48"/>
-      <c r="K41" s="48">
+      <c r="J41" s="42"/>
+      <c r="K41" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L41" s="48" t="str">
+      <c r="L41" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
@@ -2689,12 +2748,12 @@
       <c r="G42" s="4"/>
       <c r="H42" s="10"/>
       <c r="I42" s="4"/>
-      <c r="J42" s="48"/>
-      <c r="K42" s="48">
+      <c r="J42" s="42"/>
+      <c r="K42" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L42" s="48" t="str">
+      <c r="L42" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
@@ -2721,12 +2780,12 @@
       <c r="G43" s="4"/>
       <c r="H43" s="10"/>
       <c r="I43" s="4"/>
-      <c r="J43" s="48"/>
-      <c r="K43" s="48">
+      <c r="J43" s="42"/>
+      <c r="K43" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L43" s="48" t="str">
+      <c r="L43" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
@@ -2748,17 +2807,17 @@
       <c r="B44" s="6"/>
       <c r="C44" s="6"/>
       <c r="D44" s="6"/>
-      <c r="E44" s="32"/>
+      <c r="E44" s="30"/>
       <c r="F44" s="13"/>
       <c r="G44" s="4"/>
       <c r="H44" s="10"/>
       <c r="I44" s="4"/>
-      <c r="J44" s="48"/>
-      <c r="K44" s="48">
+      <c r="J44" s="42"/>
+      <c r="K44" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L44" s="48" t="str">
+      <c r="L44" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
@@ -2785,12 +2844,12 @@
       <c r="G45" s="4"/>
       <c r="H45" s="10"/>
       <c r="I45" s="4"/>
-      <c r="J45" s="48"/>
-      <c r="K45" s="48">
+      <c r="J45" s="42"/>
+      <c r="K45" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L45" s="48" t="str">
+      <c r="L45" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
@@ -2817,12 +2876,12 @@
       <c r="G46" s="4"/>
       <c r="H46" s="10"/>
       <c r="I46" s="4"/>
-      <c r="J46" s="48"/>
-      <c r="K46" s="48">
+      <c r="J46" s="42"/>
+      <c r="K46" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L46" s="48" t="str">
+      <c r="L46" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
@@ -2849,12 +2908,12 @@
       <c r="G47" s="4"/>
       <c r="H47" s="10"/>
       <c r="I47" s="4"/>
-      <c r="J47" s="48"/>
-      <c r="K47" s="48">
+      <c r="J47" s="42"/>
+      <c r="K47" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L47" s="48" t="str">
+      <c r="L47" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
@@ -2881,12 +2940,12 @@
       <c r="G48" s="4"/>
       <c r="H48" s="10"/>
       <c r="I48" s="4"/>
-      <c r="J48" s="48"/>
-      <c r="K48" s="48">
+      <c r="J48" s="42"/>
+      <c r="K48" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L48" s="48" t="str">
+      <c r="L48" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
@@ -2913,12 +2972,12 @@
       <c r="G49" s="4"/>
       <c r="H49" s="10"/>
       <c r="I49" s="4"/>
-      <c r="J49" s="48"/>
-      <c r="K49" s="48">
+      <c r="J49" s="42"/>
+      <c r="K49" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L49" s="48" t="str">
+      <c r="L49" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
@@ -2945,12 +3004,12 @@
       <c r="G50" s="4"/>
       <c r="H50" s="10"/>
       <c r="I50" s="4"/>
-      <c r="J50" s="48"/>
-      <c r="K50" s="48">
+      <c r="J50" s="42"/>
+      <c r="K50" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L50" s="48" t="str">
+      <c r="L50" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
@@ -2977,12 +3036,12 @@
       <c r="G51" s="4"/>
       <c r="H51" s="10"/>
       <c r="I51" s="4"/>
-      <c r="J51" s="48"/>
-      <c r="K51" s="48">
+      <c r="J51" s="42"/>
+      <c r="K51" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L51" s="48" t="str">
+      <c r="L51" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
@@ -3009,12 +3068,12 @@
       <c r="G52" s="4"/>
       <c r="H52" s="10"/>
       <c r="I52" s="4"/>
-      <c r="J52" s="48"/>
-      <c r="K52" s="48">
+      <c r="J52" s="42"/>
+      <c r="K52" s="42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L52" s="48" t="str">
+      <c r="L52" s="42" t="str">
         <f t="shared" si="3"/>
         <v>không thực tập</v>
       </c>
@@ -3032,188 +3091,188 @@
       </c>
     </row>
     <row r="63" spans="1:21">
-      <c r="I63" s="57" t="s">
+      <c r="I63" s="51" t="s">
         <v>158</v>
       </c>
-      <c r="J63" s="57"/>
-      <c r="K63" s="57"/>
-      <c r="L63" s="57"/>
+      <c r="J63" s="51"/>
+      <c r="K63" s="51"/>
+      <c r="L63" s="51"/>
     </row>
     <row r="64" spans="1:21">
-      <c r="I64" s="50" t="s">
+      <c r="I64" s="44" t="s">
         <v>159</v>
       </c>
-      <c r="J64" s="50" t="s">
+      <c r="J64" s="44" t="s">
         <v>160</v>
       </c>
-      <c r="K64" s="50" t="s">
+      <c r="K64" s="44" t="s">
         <v>161</v>
       </c>
-      <c r="L64" s="50" t="s">
+      <c r="L64" s="44" t="s">
         <v>175</v>
       </c>
-      <c r="M64" s="53" t="s">
+      <c r="M64" s="47" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="65" spans="9:15" ht="15.6">
-      <c r="I65" s="51">
-        <v>0</v>
-      </c>
-      <c r="J65" s="51">
-        <v>0</v>
-      </c>
-      <c r="K65" s="51" t="s">
+      <c r="I65" s="45">
+        <v>0</v>
+      </c>
+      <c r="J65" s="45">
+        <v>0</v>
+      </c>
+      <c r="K65" s="45" t="s">
         <v>162</v>
       </c>
-      <c r="L65" s="51" t="s">
+      <c r="L65" s="45" t="s">
         <v>174</v>
       </c>
       <c r="M65">
         <f>COUNTIF($L$3:$L$52,L65)</f>
         <v>50</v>
       </c>
-      <c r="N65" s="54">
+      <c r="N65" s="48">
         <f>M65/$M$72</f>
         <v>1</v>
       </c>
     </row>
     <row r="66" spans="9:15" ht="15.6">
-      <c r="I66" s="51">
+      <c r="I66" s="45">
         <v>4</v>
       </c>
-      <c r="J66" s="51">
+      <c r="J66" s="45">
         <v>1</v>
       </c>
-      <c r="K66" s="51" t="s">
+      <c r="K66" s="45" t="s">
         <v>163</v>
       </c>
-      <c r="L66" s="51" t="s">
+      <c r="L66" s="45" t="s">
         <v>173</v>
       </c>
       <c r="M66">
         <f t="shared" ref="M66:M71" si="4">COUNTIF($L$3:$L$52,L66)</f>
         <v>0</v>
       </c>
-      <c r="N66" s="54">
+      <c r="N66" s="48">
         <f t="shared" ref="N66:N71" si="5">M66/$M$72</f>
         <v>0</v>
       </c>
     </row>
     <row r="67" spans="9:15" ht="15.6">
-      <c r="I67" s="51">
+      <c r="I67" s="45">
         <v>5</v>
       </c>
-      <c r="J67" s="51">
+      <c r="J67" s="45">
         <v>2</v>
       </c>
-      <c r="K67" s="51" t="s">
+      <c r="K67" s="45" t="s">
         <v>155</v>
       </c>
-      <c r="L67" s="51" t="s">
+      <c r="L67" s="45" t="s">
         <v>172</v>
       </c>
       <c r="M67">
         <f>COUNTIF($L$3:$L$52,L67)</f>
         <v>0</v>
       </c>
-      <c r="N67" s="54">
+      <c r="N67" s="48">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="68" spans="9:15" ht="15.6">
-      <c r="I68" s="52">
+      <c r="I68" s="46">
         <v>6.5</v>
       </c>
-      <c r="J68" s="52">
+      <c r="J68" s="46">
         <v>2.5</v>
       </c>
-      <c r="K68" s="52" t="s">
+      <c r="K68" s="46" t="s">
         <v>164</v>
       </c>
-      <c r="L68" s="51" t="s">
+      <c r="L68" s="45" t="s">
         <v>171</v>
       </c>
       <c r="M68">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N68" s="54">
+      <c r="N68" s="48">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="O68" s="55">
+      <c r="O68" s="49">
         <f>SUM(N67:N68)</f>
         <v>0</v>
       </c>
     </row>
     <row r="69" spans="9:15" ht="15.6">
-      <c r="I69" s="52">
+      <c r="I69" s="46">
         <v>7</v>
       </c>
-      <c r="J69" s="52">
+      <c r="J69" s="46">
         <v>3</v>
       </c>
-      <c r="K69" s="52" t="s">
+      <c r="K69" s="46" t="s">
         <v>165</v>
       </c>
-      <c r="L69" s="51" t="s">
+      <c r="L69" s="45" t="s">
         <v>170</v>
       </c>
       <c r="M69">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N69" s="54">
+      <c r="N69" s="48">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="O69" s="55">
+      <c r="O69" s="49">
         <f>SUM(N69:N71)</f>
         <v>0</v>
       </c>
     </row>
     <row r="70" spans="9:15" ht="15.6">
-      <c r="I70" s="52">
+      <c r="I70" s="46">
         <v>8</v>
       </c>
-      <c r="J70" s="52">
+      <c r="J70" s="46">
         <v>3.5</v>
       </c>
-      <c r="K70" s="52" t="s">
+      <c r="K70" s="46" t="s">
         <v>166</v>
       </c>
-      <c r="L70" s="51" t="s">
+      <c r="L70" s="45" t="s">
         <v>169</v>
       </c>
       <c r="M70">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N70" s="54">
+      <c r="N70" s="48">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="71" spans="9:15" ht="15.6">
-      <c r="I71" s="52">
+      <c r="I71" s="46">
         <v>8.5</v>
       </c>
-      <c r="J71" s="52">
+      <c r="J71" s="46">
         <v>4</v>
       </c>
-      <c r="K71" s="52" t="s">
+      <c r="K71" s="46" t="s">
         <v>167</v>
       </c>
-      <c r="L71" s="51" t="s">
+      <c r="L71" s="45" t="s">
         <v>168</v>
       </c>
       <c r="M71">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N71" s="54">
+      <c r="N71" s="48">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -3245,784 +3304,791 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E52"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
-    <col min="2" max="2" width="28.8984375" customWidth="1"/>
-    <col min="3" max="3" width="14.296875" customWidth="1"/>
-    <col min="4" max="4" width="61.59765625" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="91.59765625" style="27" customWidth="1"/>
-    <col min="7" max="7" width="18.69921875" customWidth="1"/>
+    <col min="1" max="1" width="9" style="65"/>
+    <col min="2" max="2" width="28.8984375" style="65" customWidth="1"/>
+    <col min="3" max="3" width="14.296875" style="65" customWidth="1"/>
+    <col min="4" max="4" width="61.59765625" style="65" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="91.59765625" style="66" customWidth="1"/>
+    <col min="6" max="6" width="9" style="65"/>
+    <col min="7" max="7" width="18.69921875" style="65" customWidth="1"/>
+    <col min="8" max="16384" width="9" style="65"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" ht="39.75" customHeight="1">
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
+    <row r="1" spans="1:5" s="64" customFormat="1" ht="39.75" customHeight="1">
+      <c r="A1" s="67" t="s">
+        <v>177</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
     </row>
     <row r="2" spans="1:5" ht="35.85" customHeight="1">
-      <c r="A2" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="30" t="s">
+      <c r="A2" s="52" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="52" t="s">
         <v>94</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="E2" s="54" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A3" s="4">
+      <c r="A3" s="55">
         <v>1</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="56" t="s">
         <v>109</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D3" s="13"/>
-      <c r="E3" s="8" t="s">
+      <c r="D3" s="57"/>
+      <c r="E3" s="58" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A4" s="4">
+      <c r="A4" s="55">
         <v>2</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="56" t="s">
         <v>133</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D4" s="13"/>
-      <c r="E4" s="8" t="s">
+      <c r="D4" s="57"/>
+      <c r="E4" s="58" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A5" s="4">
+      <c r="A5" s="55">
         <v>3</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="56" t="s">
         <v>125</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D5" s="13"/>
-      <c r="E5" s="8" t="s">
+      <c r="D5" s="57"/>
+      <c r="E5" s="58" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A6" s="4">
+      <c r="A6" s="55">
         <v>4</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="56" t="s">
         <v>132</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D6" s="13"/>
-      <c r="E6" s="8" t="s">
+      <c r="D6" s="57"/>
+      <c r="E6" s="58" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A7" s="4">
+      <c r="A7" s="55">
         <v>5</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="56" t="s">
         <v>135</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="13"/>
-      <c r="E7" s="8" t="s">
+      <c r="D7" s="57"/>
+      <c r="E7" s="58" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A8" s="4">
+      <c r="A8" s="55">
         <v>6</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="56" t="s">
         <v>107</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="13"/>
-      <c r="E8" s="8" t="s">
+      <c r="D8" s="57"/>
+      <c r="E8" s="58" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A9" s="4">
+      <c r="A9" s="55">
         <v>7</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="56" t="s">
         <v>134</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D9" s="13"/>
-      <c r="E9" s="8" t="s">
+      <c r="D9" s="57"/>
+      <c r="E9" s="58" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A10" s="4">
+      <c r="A10" s="55">
         <v>8</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="56" t="s">
         <v>111</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D10" s="13"/>
-      <c r="E10" s="8" t="s">
+      <c r="D10" s="57"/>
+      <c r="E10" s="58" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A11" s="4">
+      <c r="A11" s="55">
         <v>9</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="56" t="s">
         <v>118</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="13"/>
-      <c r="E11" s="8" t="s">
+      <c r="D11" s="57"/>
+      <c r="E11" s="58" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A12" s="4">
+      <c r="A12" s="55">
         <v>10</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="56" t="s">
         <v>122</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D12" s="13"/>
-      <c r="E12" s="8" t="s">
+      <c r="D12" s="57"/>
+      <c r="E12" s="58" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A13" s="4">
+      <c r="A13" s="55">
         <v>11</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="56" t="s">
         <v>126</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D13" s="13"/>
-      <c r="E13" s="6" t="s">
+      <c r="D13" s="57"/>
+      <c r="E13" s="56" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A14" s="4">
+      <c r="A14" s="55">
         <v>12</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="56" t="s">
         <v>102</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="13"/>
-      <c r="E14" s="8" t="s">
+      <c r="D14" s="57"/>
+      <c r="E14" s="58" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A15" s="4">
+      <c r="A15" s="55">
         <v>13</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="56" t="s">
         <v>106</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D15" s="13"/>
-      <c r="E15" s="8" t="s">
+      <c r="D15" s="57"/>
+      <c r="E15" s="58" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A16" s="4">
+      <c r="A16" s="55">
         <v>14</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="56" t="s">
         <v>137</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D16" s="13"/>
-      <c r="E16" s="8" t="s">
+      <c r="D16" s="57"/>
+      <c r="E16" s="58" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A17" s="4">
+      <c r="A17" s="55">
         <v>15</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="56" t="s">
         <v>99</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="13"/>
-      <c r="E17" s="8" t="s">
+      <c r="D17" s="57"/>
+      <c r="E17" s="58" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A18" s="4">
+      <c r="A18" s="55">
         <v>16</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="56" t="s">
         <v>96</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D18" s="13"/>
-      <c r="E18" s="8" t="s">
+      <c r="D18" s="57"/>
+      <c r="E18" s="58" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A19" s="4">
+      <c r="A19" s="55">
         <v>17</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="56" t="s">
         <v>112</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="13"/>
-      <c r="E19" s="8" t="s">
+      <c r="D19" s="57"/>
+      <c r="E19" s="58" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A20" s="4">
+      <c r="A20" s="55">
         <v>18</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="56" t="s">
         <v>139</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D20" s="13"/>
-      <c r="E20" s="8" t="s">
+      <c r="D20" s="57"/>
+      <c r="E20" s="58" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A21" s="4">
+      <c r="A21" s="55">
         <v>19</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="56" t="s">
         <v>93</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="56" t="s">
         <v>52</v>
       </c>
-      <c r="D21" s="13"/>
-      <c r="E21" s="8" t="s">
+      <c r="D21" s="57"/>
+      <c r="E21" s="58" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A22" s="4">
+      <c r="A22" s="55">
         <v>20</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="56" t="s">
         <v>91</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="56" t="s">
         <v>52</v>
       </c>
-      <c r="D22" s="13"/>
-      <c r="E22" s="8" t="s">
+      <c r="D22" s="57"/>
+      <c r="E22" s="58" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A23" s="4">
+      <c r="A23" s="55">
         <v>21</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="56" t="s">
         <v>129</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D23" s="13"/>
-      <c r="E23" s="8" t="s">
+      <c r="D23" s="57"/>
+      <c r="E23" s="58" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A24" s="4">
+      <c r="A24" s="55">
         <v>22</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="56" t="s">
         <v>90</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D24" s="13"/>
-      <c r="E24" s="8" t="s">
+      <c r="D24" s="57"/>
+      <c r="E24" s="58" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A25" s="4">
+      <c r="A25" s="55">
         <v>23</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="56" t="s">
         <v>140</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D25" s="13"/>
-      <c r="E25" s="8" t="s">
+      <c r="D25" s="57"/>
+      <c r="E25" s="58" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A26" s="4">
+      <c r="A26" s="55">
         <v>24</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="56" t="s">
         <v>100</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D26" s="13"/>
-      <c r="E26" s="8" t="s">
+      <c r="D26" s="57"/>
+      <c r="E26" s="58" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A27" s="4">
+      <c r="A27" s="55">
         <v>25</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="56" t="s">
         <v>104</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D27" s="13"/>
-      <c r="E27" s="8" t="s">
+      <c r="D27" s="57"/>
+      <c r="E27" s="58" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A28" s="4">
+      <c r="A28" s="55">
         <v>26</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="56" t="s">
         <v>130</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D28" s="13"/>
-      <c r="E28" s="8" t="s">
+      <c r="D28" s="57"/>
+      <c r="E28" s="58" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A29" s="4">
+      <c r="A29" s="55">
         <v>27</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="56" t="s">
         <v>105</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="8" t="s">
+      <c r="D29" s="57"/>
+      <c r="E29" s="58" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A30" s="4">
+      <c r="A30" s="55">
         <v>28</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="56" t="s">
         <v>121</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D30" s="13"/>
-      <c r="E30" s="8" t="s">
+      <c r="D30" s="57"/>
+      <c r="E30" s="58" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A31" s="4">
+      <c r="A31" s="55">
         <v>29</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="56" t="s">
         <v>101</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D31" s="13"/>
-      <c r="E31" s="8" t="s">
+      <c r="D31" s="57"/>
+      <c r="E31" s="58" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A32" s="4">
+      <c r="A32" s="55">
         <v>30</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="56" t="s">
         <v>124</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D32" s="13"/>
-      <c r="E32" s="8" t="s">
+      <c r="D32" s="57"/>
+      <c r="E32" s="58" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A33" s="4">
+      <c r="A33" s="55">
         <v>31</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D33" s="13"/>
-      <c r="E33" s="8" t="s">
+      <c r="D33" s="57"/>
+      <c r="E33" s="58" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A34" s="4">
+      <c r="A34" s="55">
         <v>32</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="56" t="s">
         <v>115</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="C34" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D34" s="13"/>
-      <c r="E34" s="8" t="s">
+      <c r="D34" s="57"/>
+      <c r="E34" s="58" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A35" s="4">
+      <c r="A35" s="55">
         <v>33</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="56" t="s">
         <v>128</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="C35" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8" t="s">
+      <c r="D35" s="58"/>
+      <c r="E35" s="58" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A36" s="4">
+      <c r="A36" s="55">
         <v>34</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="56" t="s">
         <v>120</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="C36" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D36" s="13"/>
-      <c r="E36" s="8" t="s">
+      <c r="D36" s="57"/>
+      <c r="E36" s="58" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A37" s="4">
+      <c r="A37" s="55">
         <v>35</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="56" t="s">
         <v>95</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="C37" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D37" s="13"/>
-      <c r="E37" s="8" t="s">
+      <c r="D37" s="57"/>
+      <c r="E37" s="58" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A38" s="4">
+      <c r="A38" s="55">
         <v>36</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="56" t="s">
         <v>131</v>
       </c>
-      <c r="C38" s="6" t="s">
+      <c r="C38" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D38" s="13"/>
-      <c r="E38" s="8" t="s">
+      <c r="D38" s="57"/>
+      <c r="E38" s="58" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A39" s="4">
+      <c r="A39" s="55">
         <v>37</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="56" t="s">
         <v>117</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="C39" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D39" s="13"/>
-      <c r="E39" s="8" t="s">
+      <c r="D39" s="57"/>
+      <c r="E39" s="58" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A40" s="4">
+      <c r="A40" s="55">
         <v>38</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="56" t="s">
         <v>138</v>
       </c>
-      <c r="C40" s="6" t="s">
+      <c r="C40" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D40" s="13"/>
-      <c r="E40" s="8" t="s">
+      <c r="D40" s="57"/>
+      <c r="E40" s="58" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A41" s="4">
+      <c r="A41" s="55">
         <v>39</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="56" t="s">
         <v>92</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="56" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="13"/>
-      <c r="E41" s="8" t="s">
+      <c r="D41" s="57"/>
+      <c r="E41" s="58" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A42" s="4">
+      <c r="A42" s="55">
         <v>40</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="56" t="s">
         <v>110</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="C42" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D42" s="13"/>
-      <c r="E42" s="8" t="s">
+      <c r="D42" s="57"/>
+      <c r="E42" s="58" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A43" s="4">
+      <c r="A43" s="55">
         <v>41</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="56" t="s">
         <v>113</v>
       </c>
-      <c r="C43" s="6" t="s">
+      <c r="C43" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D43" s="13"/>
-      <c r="E43" s="8" t="s">
+      <c r="D43" s="57"/>
+      <c r="E43" s="58" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A44" s="39">
+      <c r="A44" s="59">
         <v>42</v>
       </c>
-      <c r="B44" s="40" t="s">
+      <c r="B44" s="60" t="s">
         <v>114</v>
       </c>
-      <c r="C44" s="40" t="s">
+      <c r="C44" s="60" t="s">
         <v>50</v>
       </c>
-      <c r="D44" s="41"/>
-      <c r="E44" s="42" t="s">
+      <c r="D44" s="61"/>
+      <c r="E44" s="62" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A45" s="4">
+      <c r="A45" s="55">
         <v>43</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="56" t="s">
         <v>119</v>
       </c>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D45" s="13"/>
-      <c r="E45" s="8" t="s">
+      <c r="D45" s="57"/>
+      <c r="E45" s="58" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A46" s="4">
+      <c r="A46" s="55">
         <v>44</v>
       </c>
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="56" t="s">
         <v>123</v>
       </c>
-      <c r="C46" s="6" t="s">
+      <c r="C46" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D46" s="13"/>
-      <c r="E46" s="8" t="s">
+      <c r="D46" s="57"/>
+      <c r="E46" s="58" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A47" s="4">
+      <c r="A47" s="55">
         <v>45</v>
       </c>
-      <c r="B47" s="6" t="s">
+      <c r="B47" s="56" t="s">
         <v>108</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="C47" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D47" s="13"/>
-      <c r="E47" s="8" t="s">
+      <c r="D47" s="57"/>
+      <c r="E47" s="58" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A48" s="4">
+      <c r="A48" s="55">
         <v>46</v>
       </c>
-      <c r="B48" s="6" t="s">
+      <c r="B48" s="56" t="s">
         <v>136</v>
       </c>
-      <c r="C48" s="6" t="s">
+      <c r="C48" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D48" s="13"/>
-      <c r="E48" s="28" t="s">
+      <c r="D48" s="57"/>
+      <c r="E48" s="63" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A49" s="4">
+      <c r="A49" s="55">
         <v>47</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="56" t="s">
         <v>98</v>
       </c>
-      <c r="C49" s="6" t="s">
+      <c r="C49" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D49" s="13"/>
-      <c r="E49" s="28" t="s">
+      <c r="D49" s="57"/>
+      <c r="E49" s="63" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A50" s="4">
+      <c r="A50" s="55">
         <v>48</v>
       </c>
-      <c r="B50" s="6" t="s">
+      <c r="B50" s="56" t="s">
         <v>116</v>
       </c>
-      <c r="C50" s="6" t="s">
+      <c r="C50" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D50" s="13"/>
-      <c r="E50" s="28" t="s">
+      <c r="D50" s="57"/>
+      <c r="E50" s="63" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A51" s="4">
+      <c r="A51" s="55">
         <v>49</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="B51" s="56" t="s">
         <v>97</v>
       </c>
-      <c r="C51" s="6" t="s">
+      <c r="C51" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D51" s="13"/>
-      <c r="E51" s="28" t="s">
+      <c r="D51" s="57"/>
+      <c r="E51" s="63" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A52" s="4">
+      <c r="A52" s="55">
         <v>50</v>
       </c>
-      <c r="B52" s="6" t="s">
+      <c r="B52" s="56" t="s">
         <v>127</v>
       </c>
-      <c r="C52" s="6" t="s">
+      <c r="C52" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="D52" s="13"/>
-      <c r="E52" s="8" t="s">
+      <c r="D52" s="57"/>
+      <c r="E52" s="58" t="s">
         <v>89</v>
       </c>
     </row>
@@ -4033,7 +4099,7 @@
     <sortCondition ref="B3:B52"/>
   </sortState>
   <mergeCells count="1">
-    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4076,10 +4142,10 @@
       <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="35" t="s">
+      <c r="B2" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="35" t="s">
+      <c r="C2" s="33" t="s">
         <v>8</v>
       </c>
       <c r="D2" s="4"/>
@@ -4092,10 +4158,10 @@
       <c r="A3" s="4">
         <v>2</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="36" t="s">
+      <c r="C3" s="34" t="s">
         <v>18</v>
       </c>
       <c r="D3" s="4"/>
@@ -4108,10 +4174,10 @@
       <c r="A4" s="4">
         <v>3</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="34" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="4">
@@ -4126,10 +4192,10 @@
       <c r="A5" s="4">
         <v>4</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="35" t="s">
+      <c r="C5" s="33" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="10">
@@ -4144,10 +4210,10 @@
       <c r="A6" s="4">
         <v>5</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="36" t="s">
+      <c r="C6" s="34" t="s">
         <v>25</v>
       </c>
       <c r="D6" s="10">
@@ -4162,10 +4228,10 @@
       <c r="A7" s="4">
         <v>6</v>
       </c>
-      <c r="B7" s="36" t="s">
+      <c r="B7" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="36" t="s">
+      <c r="C7" s="34" t="s">
         <v>11</v>
       </c>
       <c r="D7" s="10">
@@ -4180,10 +4246,10 @@
       <c r="A8" s="4">
         <v>8</v>
       </c>
-      <c r="B8" s="36" t="s">
+      <c r="B8" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="36" t="s">
+      <c r="C8" s="34" t="s">
         <v>28</v>
       </c>
       <c r="D8" s="10"/>
@@ -4194,10 +4260,10 @@
       <c r="A9" s="4">
         <v>9</v>
       </c>
-      <c r="B9" s="36" t="s">
+      <c r="B9" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="37" t="s">
+      <c r="C9" s="35" t="s">
         <v>29</v>
       </c>
       <c r="D9" s="10">
@@ -4210,10 +4276,10 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="4"/>
-      <c r="B10" s="36" t="s">
+      <c r="B10" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="C10" s="37"/>
+      <c r="C10" s="35"/>
       <c r="D10" s="10">
         <v>6</v>
       </c>
@@ -4226,10 +4292,10 @@
       <c r="A11" s="4">
         <v>10</v>
       </c>
-      <c r="B11" s="36" t="s">
+      <c r="B11" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="36"/>
+      <c r="C11" s="34"/>
       <c r="D11" s="10"/>
       <c r="E11" s="20"/>
       <c r="F11" s="7" t="s">
@@ -4240,10 +4306,10 @@
       <c r="A12" s="4">
         <v>11</v>
       </c>
-      <c r="B12" s="36" t="s">
+      <c r="B12" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="36" t="s">
+      <c r="C12" s="34" t="s">
         <v>41</v>
       </c>
       <c r="D12" s="10">
@@ -4256,10 +4322,10 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="4"/>
-      <c r="B13" s="36" t="s">
+      <c r="B13" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="36" t="s">
+      <c r="C13" s="34" t="s">
         <v>57</v>
       </c>
       <c r="D13" s="10">
@@ -4272,10 +4338,10 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="4"/>
-      <c r="B14" s="36" t="s">
+      <c r="B14" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="C14" s="36" t="s">
+      <c r="C14" s="34" t="s">
         <v>59</v>
       </c>
       <c r="D14" s="10">
@@ -4290,10 +4356,10 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="4"/>
-      <c r="B15" s="36" t="s">
+      <c r="B15" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="C15" s="36" t="s">
+      <c r="C15" s="34" t="s">
         <v>62</v>
       </c>
       <c r="D15" s="10">
@@ -4308,10 +4374,10 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="4"/>
-      <c r="B16" s="36" t="s">
+      <c r="B16" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="C16" s="36" t="s">
+      <c r="C16" s="34" t="s">
         <v>64</v>
       </c>
       <c r="D16" s="10">
@@ -4324,10 +4390,10 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="4"/>
-      <c r="B17" s="36" t="s">
+      <c r="B17" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="C17" s="36" t="s">
+      <c r="C17" s="34" t="s">
         <v>72</v>
       </c>
       <c r="D17" s="10">
@@ -4340,10 +4406,10 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="4"/>
-      <c r="B18" s="36" t="s">
+      <c r="B18" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="C18" s="36"/>
+      <c r="C18" s="34"/>
       <c r="D18" s="10">
         <v>3</v>
       </c>
@@ -4354,20 +4420,20 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="4"/>
-      <c r="B19" s="36" t="s">
+      <c r="B19" s="34" t="s">
         <v>78</v>
       </c>
-      <c r="C19" s="36"/>
+      <c r="C19" s="34"/>
       <c r="D19" s="10"/>
       <c r="E19" s="19"/>
       <c r="F19" s="4"/>
     </row>
     <row r="20" spans="1:7" ht="33.6">
       <c r="A20" s="4"/>
-      <c r="B20" s="38" t="s">
+      <c r="B20" s="36" t="s">
         <v>77</v>
       </c>
-      <c r="C20" s="38" t="s">
+      <c r="C20" s="36" t="s">
         <v>74</v>
       </c>
       <c r="D20" s="10">
@@ -4380,10 +4446,10 @@
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="4"/>
-      <c r="B21" s="38" t="s">
+      <c r="B21" s="36" t="s">
         <v>79</v>
       </c>
-      <c r="C21" s="38" t="s">
+      <c r="C21" s="36" t="s">
         <v>80</v>
       </c>
       <c r="D21" s="10">
@@ -4394,10 +4460,10 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4"/>
-      <c r="B22" s="38" t="s">
+      <c r="B22" s="36" t="s">
         <v>81</v>
       </c>
-      <c r="C22" s="38" t="s">
+      <c r="C22" s="36" t="s">
         <v>82</v>
       </c>
       <c r="D22" s="10">
@@ -4408,10 +4474,10 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4"/>
-      <c r="B23" s="36" t="s">
+      <c r="B23" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="C23" s="38" t="s">
+      <c r="C23" s="36" t="s">
         <v>84</v>
       </c>
       <c r="D23" s="10">
@@ -4422,10 +4488,10 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4"/>
-      <c r="B24" s="36" t="s">
+      <c r="B24" s="34" t="s">
         <v>85</v>
       </c>
-      <c r="C24" s="38" t="s">
+      <c r="C24" s="36" t="s">
         <v>86</v>
       </c>
       <c r="D24" s="10">

</xml_diff>